<commit_message>
Add outlet sheet support for Crestron switches
</commit_message>
<xml_diff>
--- a/HA设备接口配置表.xlsx
+++ b/HA设备接口配置表.xlsx
@@ -11,6 +11,7 @@
     <sheet name="灯光" sheetId="1" r:id="rId2"/>
     <sheet name="空调" sheetId="3" r:id="rId3"/>
     <sheet name="窗帘" sheetId="2" r:id="rId4"/>
+    <sheet name="插座" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">灯光!$A$1:$I$8</definedName>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="55">
   <si>
     <t>灯光</t>
   </si>
@@ -44,6 +45,12 @@
 4.双色温类型的由模拟量的join控制，分别有亮度join和色温join，亮度值范围0-65535，色温值范围2700-6500.</t>
   </si>
   <si>
+    <t>插座</t>
+  </si>
+  <si>
+    <t>数字量的join控制，开是1个join，关是1个join</t>
+  </si>
+  <si>
     <t>空调</t>
   </si>
   <si>
@@ -174,6 +181,30 @@
   </si>
   <si>
     <t>布帘1</t>
+  </si>
+  <si>
+    <t>落地灯</t>
+  </si>
+  <si>
+    <t>台灯</t>
+  </si>
+  <si>
+    <t>1F</t>
+  </si>
+  <si>
+    <t>书房</t>
+  </si>
+  <si>
+    <t>儿子房</t>
+  </si>
+  <si>
+    <t>客卫玄关</t>
+  </si>
+  <si>
+    <t>2F</t>
+  </si>
+  <si>
+    <t>休闲区</t>
   </si>
 </sst>
 </file>
@@ -186,10 +217,16 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="WPSLingXiuHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="WPSLingXiuHei"/>
       <charset val="134"/>
     </font>
@@ -718,159 +755,168 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyBorder="1">
@@ -1413,38 +1459,46 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B2:C10"/>
+  <dimension ref="B2:C11"/>
   <sheetFormatPr defaultColWidth="7.83088235294118" defaultRowHeight="16.8" outlineLevelCol="2"/>
   <cols>
     <col min="3" max="3" width="112.360294117647" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" ht="99" customHeight="1" spans="2:3">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" ht="99" customHeight="1" spans="2:3">
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" ht="99" customHeight="1" spans="2:3">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="2:3">
-      <c r="C10" s="7"/>
+    <row r="5" ht="99" customHeight="1" spans="2:3">
+      <c r="B5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3">
+      <c r="C11" s="10"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertRows="0" insertColumns="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
@@ -1470,31 +1524,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -1502,16 +1556,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -1525,16 +1579,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F3">
         <v>2</v>
@@ -1548,16 +1602,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
         <v>20</v>
-      </c>
-      <c r="E4" t="s">
-        <v>18</v>
       </c>
       <c r="F4">
         <v>3</v>
@@ -1571,16 +1625,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F5">
         <v>4</v>
@@ -1591,16 +1645,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F6">
         <v>5</v>
@@ -1611,16 +1665,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -1634,16 +1688,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H8">
         <v>3</v>
@@ -1675,52 +1729,52 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="L1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="M1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="O1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:16">
@@ -1728,10 +1782,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D2">
         <v>505</v>
@@ -1778,10 +1832,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D3">
         <v>490</v>
@@ -1847,28 +1901,28 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -1876,13 +1930,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E2">
         <v>700</v>
@@ -1902,13 +1956,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E3">
         <v>704</v>
@@ -1928,13 +1982,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" t="s">
         <v>43</v>
-      </c>
-      <c r="D4" t="s">
-        <v>41</v>
       </c>
       <c r="E4">
         <v>708</v>
@@ -1954,13 +2008,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E5">
         <v>712</v>
@@ -1979,6 +2033,218 @@
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertRows="0" insertColumns="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultColWidth="8.94117647058824" defaultRowHeight="16.8" outlineLevelCol="5"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="1">
+        <v>147</v>
+      </c>
+      <c r="F2" s="1">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" s="1">
+        <v>149</v>
+      </c>
+      <c r="F3" s="1">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="1">
+        <v>151</v>
+      </c>
+      <c r="F4" s="1">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="1">
+        <v>153</v>
+      </c>
+      <c r="F5" s="1">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="1">
+        <v>155</v>
+      </c>
+      <c r="F6" s="1">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="1">
+        <v>157</v>
+      </c>
+      <c r="F7" s="1">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="1">
+        <v>159</v>
+      </c>
+      <c r="F8" s="1">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" s="1">
+        <v>161</v>
+      </c>
+      <c r="F9" s="1">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="1">
+        <v>163</v>
+      </c>
+      <c r="F10" s="1">
+        <v>164</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
 </file>

</xml_diff>